<commit_message>
Actualizacion final de documentos.
</commit_message>
<xml_diff>
--- a/proyecto-asul/fase-05-seguridad/tabla-stride-cliente.xlsx
+++ b/proyecto-asul/fase-05-seguridad/tabla-stride-cliente.xlsx
@@ -588,12 +588,12 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>No se confirmó en la entrevista si el segundo factor de autenticación (MFA) está habilitado de forma consistente en todas las cuentas.</t>
+          <t>Se confirmó directamente con el cliente que el segundo factor de autenticación (MFA) está habilitado en todas las cuentas de Microsoft 365/Azure.</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Credenciales comprometidas por phishing permitirían acceso sin una segunda barrera de verificación.</t>
+          <t>Si el MFA llegara a desactivarse o existiera una cuenta de servicio sin segundo factor y sin auditar, credenciales comprometidas por phishing permitirían acceso sin barrera adicional.</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -603,22 +603,22 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Bajo</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>Dominio corporativo propio en Entra ID (MFA sin confirmar)</t>
+          <t>MFA obligatorio habilitado en todas las cuentas de Microsoft 365/Azure (confirmado directamente con el cliente, octubre 2026)</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Confirmar y forzar MFA obligatorio en todas las cuentas de Microsoft 365 y Azure</t>
+          <t>Mantener el MFA obligatorio y auditar periódicamente que no existan cuentas de servicio o excepciones sin segundo factor</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -628,7 +628,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Pendiente de confirmar</t>
+          <t>Mitigado / Cerrado</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Correccion en mal entendido de JIRA
</commit_message>
<xml_diff>
--- a/proyecto-asul/fase-05-seguridad/tabla-stride-cliente.xlsx
+++ b/proyecto-asul/fase-05-seguridad/tabla-stride-cliente.xlsx
@@ -516,7 +516,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Azure DevOps (Azure Boards) - usuario compartido</t>
+          <t>Jira (cliente) - cuenta compartida</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -526,12 +526,12 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>El cliente entregó una sola licencia/usuario (el de Alejandro); todo el lado de Asul accede con esa misma cuenta, sin usuarios individuales.</t>
+          <t>El cliente entregó una sola licencia/usuario de Jira (el de Alejandro); todo el lado de soporte de Asul accede al Jira del cliente con esa misma cuenta para consultar y actualizar tickets. En Azure DevOps no ocurre esto: cada persona del equipo de Asul ya tiene su propia cuenta individual con permisos designados.</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Una acción o cambio erróneo en un ticket no puede atribuirse a una persona específica; si las credenciales se filtran, cualquiera actúa como el líder técnico autorizado.</t>
+          <t>Una consulta o actualización errónea de un ticket en Jira no puede atribuirse a una persona específica; si las credenciales de Jira se filtran, cualquiera actúa en el Jira del cliente como el líder técnico autorizado.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -551,12 +551,12 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Ninguno reportado más allá de la licencia entregada por el cliente</t>
+          <t>Ninguno reportado más allá de la licencia de Jira entregada por el cliente</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Solicitar cuentas nombradas o acceso federado/invitado al cliente; en su defecto, llevar bitácora interna de uso de la cuenta compartida</t>
+          <t>Solicitar al cliente licencias/cuentas nombradas de Jira o acceso federado/invitado; en su defecto, llevar bitácora interna de uso de la cuenta de Jira compartida</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">

</xml_diff>